<commit_message>
Add July budget explanation and email draft
Co-authored-by: peterli0913 <peterli0913@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/2026/PP-2607 Monthly Budget Application Form - PP Annual Shutdown Works -V2.xlsx
+++ b/2026/PP-2607 Monthly Budget Application Form - PP Annual Shutdown Works -V2.xlsx
@@ -6058,7 +6058,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="FFFF0000"/>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -6147,12 +6147,12 @@
         <v>0</v>
       </c>
       <c r="E4" s="169">
-        <f>SUMIFS('K(Cost center)-Opex (Service)'!$S:$S,'K(Cost center)-Opex (Service)'!$D:$D,$B4,'K(Cost center)-Opex (Service)'!$X:$X,E$3)</f>
-        <v>50438.66</v>
+        <f>SUMIFS('K(Cost center)-Opex (Service)'!$O:$O,'K(Cost center)-Opex (Service)'!$D:$D,$B4,'K(Cost center)-Opex (Service)'!$X:$X,E$3)</f>
+        <v>39032.22</v>
       </c>
       <c r="F4" s="169">
-        <f>SUMIFS('K(Cost center)-Opex (Service)'!$S:$S,'K(Cost center)-Opex (Service)'!$D:$D,$B4,'K(Cost center)-Opex (Service)'!$X:$X,F$3)</f>
-        <v>20368</v>
+        <f>SUMIFS('K(Cost center)-Opex (Service)'!$O:$O,'K(Cost center)-Opex (Service)'!$D:$D,$B4,'K(Cost center)-Opex (Service)'!$X:$X,F$3)</f>
+        <v>16973</v>
       </c>
       <c r="G4" s="169">
         <f t="shared" ref="G4:G10" si="0">SUM(C4:D4)</f>
@@ -6160,7 +6160,7 @@
       </c>
       <c r="H4" s="184">
         <f t="shared" ref="H4:H10" si="1">SUM(E4:F4)</f>
-        <v>70806.66</v>
+        <v>56005.22</v>
       </c>
     </row>
     <row r="5" customHeight="1" spans="1:8">
@@ -6177,20 +6177,20 @@
         <v>0</v>
       </c>
       <c r="E5" s="169">
-        <f>SUMIFS('K(Cost center)-Opex (Service)'!$S:$S,'K(Cost center)-Opex (Service)'!$D:$D,$B5,'K(Cost center)-Opex (Service)'!$X:$X,E$3)</f>
+        <f>SUMIFS('K(Cost center)-Opex (Service)'!$O:$O,'K(Cost center)-Opex (Service)'!$D:$D,$B5,'K(Cost center)-Opex (Service)'!$X:$X,E$3)</f>
         <v>0</v>
       </c>
       <c r="F5" s="169">
-        <f>SUMIFS('K(Cost center)-Opex (Service)'!$S:$S,'K(Cost center)-Opex (Service)'!$D:$D,$B5,'K(Cost center)-Opex (Service)'!$X:$X,F$3)</f>
-        <v>1200</v>
+        <f>SUMIFS('K(Cost center)-Opex (Service)'!$O:$O,'K(Cost center)-Opex (Service)'!$D:$D,$B5,'K(Cost center)-Opex (Service)'!$X:$X,F$3)</f>
+        <v>1000</v>
       </c>
       <c r="G5" s="169">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="H5" s="184">
-        <f t="shared" si="1"/>
-        <v>1200</v>
+        <f t="shared" si="1">SUM(E5:F5)</f>
+        <v>1000</v>
       </c>
     </row>
     <row r="6" customHeight="1" spans="1:8">
@@ -6207,11 +6207,11 @@
         <v>0</v>
       </c>
       <c r="E6" s="169">
-        <f>SUMIFS('K(Cost center)-Opex (Service)'!$S:$S,'K(Cost center)-Opex (Service)'!$D:$D,$B6,'K(Cost center)-Opex (Service)'!$X:$X,E$3)</f>
+        <f>SUMIFS('K(Cost center)-Opex (Service)'!$O:$O,'K(Cost center)-Opex (Service)'!$D:$D,$B6,'K(Cost center)-Opex (Service)'!$X:$X,E$3)</f>
         <v>0</v>
       </c>
       <c r="F6" s="169">
-        <f>SUMIFS('K(Cost center)-Opex (Service)'!$S:$S,'K(Cost center)-Opex (Service)'!$D:$D,$B6,'K(Cost center)-Opex (Service)'!$X:$X,F$3)</f>
+        <f>SUMIFS('K(Cost center)-Opex (Service)'!$O:$O,'K(Cost center)-Opex (Service)'!$D:$D,$B6,'K(Cost center)-Opex (Service)'!$X:$X,F$3)</f>
         <v>0</v>
       </c>
       <c r="G6" s="169">
@@ -6219,7 +6219,7 @@
         <v>0</v>
       </c>
       <c r="H6" s="184">
-        <f t="shared" si="1"/>
+        <f t="shared" si="1">SUM(E6:F6)</f>
         <v>0</v>
       </c>
     </row>
@@ -6237,20 +6237,20 @@
         <v>0</v>
       </c>
       <c r="E7" s="169">
-        <f>SUMIFS('K(Cost center)-Opex (Service)'!$S:$S,'K(Cost center)-Opex (Service)'!$D:$D,$B7,'K(Cost center)-Opex (Service)'!$X:$X,E$3)</f>
-        <v>3600</v>
+        <f>SUMIFS('K(Cost center)-Opex (Service)'!$O:$O,'K(Cost center)-Opex (Service)'!$D:$D,$B7,'K(Cost center)-Opex (Service)'!$X:$X,E$3)</f>
+        <v>3000</v>
       </c>
       <c r="F7" s="169">
-        <f>SUMIFS('K(Cost center)-Opex (Service)'!$S:$S,'K(Cost center)-Opex (Service)'!$D:$D,$B7,'K(Cost center)-Opex (Service)'!$X:$X,F$3)</f>
-        <v>1560</v>
+        <f>SUMIFS('K(Cost center)-Opex (Service)'!$O:$O,'K(Cost center)-Opex (Service)'!$D:$D,$B7,'K(Cost center)-Opex (Service)'!$X:$X,F$3)</f>
+        <v>1300</v>
       </c>
       <c r="G7" s="169">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="H7" s="184">
-        <f t="shared" si="1"/>
-        <v>5160</v>
+        <f t="shared" si="1">SUM(E7:F7)</f>
+        <v>4300</v>
       </c>
     </row>
     <row r="8" customHeight="1" spans="1:8">
@@ -6267,11 +6267,11 @@
         <v>0</v>
       </c>
       <c r="E8" s="169">
-        <f>SUMIFS('K(Cost center)-Opex (Service)'!$S:$S,'K(Cost center)-Opex (Service)'!$D:$D,$B8,'K(Cost center)-Opex (Service)'!$X:$X,E$3)</f>
+        <f>SUMIFS('K(Cost center)-Opex (Service)'!$O:$O,'K(Cost center)-Opex (Service)'!$D:$D,$B8,'K(Cost center)-Opex (Service)'!$X:$X,E$3)</f>
         <v>0</v>
       </c>
       <c r="F8" s="169">
-        <f>SUMIFS('K(Cost center)-Opex (Service)'!$S:$S,'K(Cost center)-Opex (Service)'!$D:$D,$B8,'K(Cost center)-Opex (Service)'!$X:$X,F$3)</f>
+        <f>SUMIFS('K(Cost center)-Opex (Service)'!$O:$O,'K(Cost center)-Opex (Service)'!$D:$D,$B8,'K(Cost center)-Opex (Service)'!$X:$X,F$3)</f>
         <v>0</v>
       </c>
       <c r="G8" s="169">
@@ -6279,7 +6279,7 @@
         <v>0</v>
       </c>
       <c r="H8" s="184">
-        <f t="shared" si="1"/>
+        <f t="shared" si="1">SUM(E8:F8)</f>
         <v>0</v>
       </c>
     </row>
@@ -6297,11 +6297,11 @@
         <v>0</v>
       </c>
       <c r="E9" s="169">
-        <f>SUMIFS('K(Cost center)-Opex (Service)'!$S:$S,'K(Cost center)-Opex (Service)'!$D:$D,$B9,'K(Cost center)-Opex (Service)'!$X:$X,E$3)</f>
-        <v>77856.76</v>
+        <f>SUMIFS('K(Cost center)-Opex (Service)'!$O:$O,'K(Cost center)-Opex (Service)'!$D:$D,$B9,'K(Cost center)-Opex (Service)'!$X:$X,E$3)</f>
+        <v>64880.63</v>
       </c>
       <c r="F9" s="169">
-        <f>SUMIFS('K(Cost center)-Opex (Service)'!$S:$S,'K(Cost center)-Opex (Service)'!$D:$D,$B9,'K(Cost center)-Opex (Service)'!$X:$X,F$3)</f>
+        <f>SUMIFS('K(Cost center)-Opex (Service)'!$O:$O,'K(Cost center)-Opex (Service)'!$D:$D,$B9,'K(Cost center)-Opex (Service)'!$X:$X,F$3)</f>
         <v>0</v>
       </c>
       <c r="G9" s="169">
@@ -6309,8 +6309,8 @@
         <v>0</v>
       </c>
       <c r="H9" s="184">
-        <f t="shared" si="1"/>
-        <v>77856.76</v>
+        <f t="shared" si="1">SUM(E9:F9)</f>
+        <v>64880.63</v>
       </c>
     </row>
     <row r="10" customHeight="1" spans="1:8">
@@ -6327,11 +6327,11 @@
         <v>0</v>
       </c>
       <c r="E10" s="169">
-        <f>SUMIFS('K(Cost center)-Opex (Service)'!$S:$S,'K(Cost center)-Opex (Service)'!$D:$D,$B10,'K(Cost center)-Opex (Service)'!$X:$X,E$3)</f>
+        <f>SUMIFS('K(Cost center)-Opex (Service)'!$O:$O,'K(Cost center)-Opex (Service)'!$D:$D,$B10,'K(Cost center)-Opex (Service)'!$X:$X,E$3)</f>
         <v>0</v>
       </c>
       <c r="F10" s="169">
-        <f>SUMIFS('K(Cost center)-Opex (Service)'!$S:$S,'K(Cost center)-Opex (Service)'!$D:$D,$B10,'K(Cost center)-Opex (Service)'!$X:$X,F$3)</f>
+        <f>SUMIFS('K(Cost center)-Opex (Service)'!$O:$O,'K(Cost center)-Opex (Service)'!$D:$D,$B10,'K(Cost center)-Opex (Service)'!$X:$X,F$3)</f>
         <v>0</v>
       </c>
       <c r="G10" s="169">
@@ -6339,7 +6339,7 @@
         <v>0</v>
       </c>
       <c r="H10" s="184">
-        <f t="shared" si="1"/>
+        <f t="shared" si="1">SUM(E10:F10)</f>
         <v>0</v>
       </c>
     </row>
@@ -6357,20 +6357,20 @@
         <v>0</v>
       </c>
       <c r="E11" s="181">
-        <f t="shared" si="2"/>
-        <v>131895.42</v>
+        <f t="shared" si="2">SUM(E4:E10)</f>
+        <v>106912.85</v>
       </c>
       <c r="F11" s="181">
-        <f t="shared" si="2"/>
-        <v>23128</v>
+        <f t="shared" si="2">SUM(F4:F10)</f>
+        <v>19273</v>
       </c>
       <c r="G11" s="180">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="H11" s="185">
-        <f t="shared" si="2"/>
-        <v>155023.42</v>
+        <f t="shared" si="2">SUM(H4:H10)</f>
+        <v>126185.85</v>
       </c>
     </row>
   </sheetData>

</xml_diff>